<commit_message>
Daily EOD data and reports for 2026-07-17
</commit_message>
<xml_diff>
--- a/asx_eod_output/Report_XLSX/Report_20260717.xlsx
+++ b/asx_eod_output/Report_XLSX/Report_20260717.xlsx
@@ -488,24 +488,24 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>1.335</v>
+        <v>1.305</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>-0.055</v>
+        <v>-0.08500000000000001</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>-3.96%</t>
+          <t>-6.12%</t>
         </is>
       </c>
       <c r="E4" s="3" t="n">
         <v>153181</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>204496.63</v>
+        <v>199901.2</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>-8424.950000000001</v>
+        <v>-13020.38</v>
       </c>
     </row>
     <row r="5">
@@ -515,24 +515,24 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>1.987</v>
+        <v>2.02</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>0.08699999999999999</v>
+        <v>0.12</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>4.58%</t>
+          <t>6.32%</t>
         </is>
       </c>
       <c r="E5" s="3" t="n">
         <v>70000</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>139090</v>
+        <v>141400</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>6090</v>
+        <v>8400</v>
       </c>
     </row>
     <row r="6">
@@ -542,24 +542,24 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>1.03</v>
+        <v>1.025</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>-0.03</v>
+        <v>-0.035</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>-2.83%</t>
+          <t>-3.30%</t>
         </is>
       </c>
       <c r="E6" s="3" t="n">
         <v>57458</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>59181.74</v>
+        <v>58894.45</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>-1723.74</v>
+        <v>-2011.03</v>
       </c>
     </row>
     <row r="7">
@@ -569,24 +569,24 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>57.35</v>
+        <v>57.54</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>-1.79</v>
+        <v>-1.6</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>-3.03%</t>
+          <t>-2.71%</t>
         </is>
       </c>
       <c r="E7" s="3" t="n">
         <v>11065</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>634577.75</v>
+        <v>636680.1</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>-19806.35</v>
+        <v>-17704</v>
       </c>
     </row>
     <row r="8">
@@ -623,14 +623,14 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>170.64</v>
+        <v>171.78</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>-2.49</v>
+        <v>-1.35</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>-1.44%</t>
+          <t>-0.78%</t>
         </is>
       </c>
       <c r="E9" s="3" t="n">
@@ -650,24 +650,24 @@
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>0.5</v>
+        <v>0.49</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>-0.035</v>
+        <v>-0.045</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>-6.54%</t>
+          <t>-8.41%</t>
         </is>
       </c>
       <c r="E10" s="3" t="n">
         <v>10000</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>5000</v>
+        <v>4900</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>-350</v>
+        <v>-450</v>
       </c>
     </row>
     <row r="11">
@@ -677,24 +677,24 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>123.94</v>
+        <v>123.32</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>1.99</v>
+        <v>1.37</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>1.63%</t>
+          <t>1.12%</t>
         </is>
       </c>
       <c r="E11" s="3" t="n">
         <v>3450</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>427593</v>
+        <v>425454</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>6865.5</v>
+        <v>4726.5</v>
       </c>
     </row>
     <row r="12">
@@ -704,24 +704,24 @@
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>0</v>
+        <v>0.235</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>-0.235</v>
+        <v>0</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>-100.00%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="E12" s="3" t="n">
         <v>20000</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>0</v>
+        <v>4700</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>-4700</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -785,24 +785,24 @@
         </is>
       </c>
       <c r="B15" s="2" t="n">
-        <v>0.105</v>
+        <v>0.1</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>0</v>
+        <v>-0.005</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>-4.76%</t>
         </is>
       </c>
       <c r="E15" s="3" t="n">
         <v>6000</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>630</v>
+        <v>600</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>0</v>
+        <v>-30</v>
       </c>
     </row>
     <row r="16">
@@ -812,14 +812,14 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>36.28</v>
+        <v>36.56</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>-0.35</v>
+        <v>-0.07000000000000001</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>-0.96%</t>
+          <t>-0.19%</t>
         </is>
       </c>
       <c r="E16" s="3" t="n">
@@ -839,24 +839,24 @@
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>30.28</v>
+        <v>30.46</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>0.79</v>
+        <v>0.97</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2.68%</t>
+          <t>3.29%</t>
         </is>
       </c>
       <c r="E17" s="3" t="n">
         <v>1288</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>39000.64</v>
+        <v>39232.48</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>1017.52</v>
+        <v>1249.36</v>
       </c>
     </row>
     <row r="18">
@@ -870,10 +870,10 @@
       <c r="D18" s="5" t="inlineStr"/>
       <c r="E18" s="7" t="inlineStr"/>
       <c r="F18" s="8" t="n">
-        <v>1510527.32</v>
+        <v>1512719.79</v>
       </c>
       <c r="G18" s="8" t="n">
-        <v>-22441.44</v>
+        <v>-20248.97</v>
       </c>
     </row>
   </sheetData>

</xml_diff>